<commit_message>
Update site for May 29 playoffs with leaderboard UX and Vercel deploy.
Add playoff_results.json as the source of truth for bracket state, a site banner, enhanced leaderboard UI, DB sync/fallback, and Next.js Vercel config so production reflects today's Stanley Cup Final matchup.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/NHL_Playoffs_2026_Bracket_Scorer.xlsx
+++ b/NHL_Playoffs_2026_Bracket_Scorer.xlsx
@@ -857,16 +857,22 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Boston Bruins</t>
+          <t>Carolina Hurricanes</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Buffalo Sabres</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
+          <t>Ottawa Senators</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Carolina Hurricanes</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="G2" s="7">
         <f>IF(E2&lt;&gt;"","Final",IF(AND(C2&lt;&gt;"",D2&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -885,16 +891,22 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Montreal Canadiens</t>
+          <t>Pittsburgh Penguins</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Tampa Bay Lightning</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
+          <t>Philadelphia Flyers</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Philadelphia Flyers</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="G3" s="7">
         <f>IF(E3&lt;&gt;"","Final",IF(AND(C3&lt;&gt;"",D3&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -913,16 +925,22 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Ottawa Senators</t>
+          <t>Buffalo Sabres</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Carolina Hurricanes</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
+          <t>Boston Bruins</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Buffalo Sabres</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="G4" s="7">
         <f>IF(E4&lt;&gt;"","Final",IF(AND(C4&lt;&gt;"",D4&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -941,16 +959,22 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Philadelphia Flyers</t>
+          <t>Tampa Bay Lightning</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Pittsburgh Penguins</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
+          <t>Montreal Canadiens</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Montreal Canadiens</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="G5" s="7">
         <f>IF(E5&lt;&gt;"","Final",IF(AND(C5&lt;&gt;"",D5&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -969,16 +993,22 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
+          <t>Colorado Avalanche</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
           <t>Los Angeles Kings</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Colorado Avalanche</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="F6" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="G6" s="7">
         <f>IF(E6&lt;&gt;"","Final",IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -997,16 +1027,22 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
+          <t>Dallas Stars</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
           <t>Minnesota Wild</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Dallas Stars</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Minnesota Wild</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="G7" s="7">
         <f>IF(E7&lt;&gt;"","Final",IF(AND(C7&lt;&gt;"",D7&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1025,16 +1061,22 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
+          <t>Vegas Golden Knights</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
           <t>Utah Mammoth</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Vegas Golden Knights</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
+      <c r="F8" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="G8" s="7">
         <f>IF(E8&lt;&gt;"","Final",IF(AND(C8&lt;&gt;"",D8&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1053,16 +1095,22 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
+          <t>Edmonton Oilers</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
           <t>Anaheim Ducks</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Edmonton Oilers</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Anaheim Ducks</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="G9" s="7">
         <f>IF(E9&lt;&gt;"","Final",IF(AND(C9&lt;&gt;"",D9&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1087,8 +1135,14 @@
         <f>IF(E3="","",E3)</f>
         <v/>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Carolina Hurricanes</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="G10" s="7">
         <f>IF(E10&lt;&gt;"","Final",IF(AND(C10&lt;&gt;"",D10&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1113,8 +1167,14 @@
         <f>IF(E5="","",E5)</f>
         <v/>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Montreal Canadiens</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="G11" s="7">
         <f>IF(E11&lt;&gt;"","Final",IF(AND(C11&lt;&gt;"",D11&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1139,8 +1199,14 @@
         <f>IF(E7="","",E7)</f>
         <v/>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Colorado Avalanche</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="G12" s="7">
         <f>IF(E12&lt;&gt;"","Final",IF(AND(C12&lt;&gt;"",D12&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1165,8 +1231,14 @@
         <f>IF(E9="","",E9)</f>
         <v/>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Vegas Golden Knights</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="G13" s="7">
         <f>IF(E13&lt;&gt;"","Final",IF(AND(C13&lt;&gt;"",D13&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1191,8 +1263,14 @@
         <f>IF(E11="","",E11)</f>
         <v/>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Carolina Hurricanes</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="G14" s="7">
         <f>IF(E14&lt;&gt;"","Final",IF(AND(C14&lt;&gt;"",D14&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>
@@ -1217,8 +1295,14 @@
         <f>IF(E13="","",E13)</f>
         <v/>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Vegas Golden Knights</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="G15" s="7">
         <f>IF(E15&lt;&gt;"","Final",IF(AND(C15&lt;&gt;"",D15&lt;&gt;""),"In Progress","Not Set"))</f>
         <v/>

</xml_diff>

<commit_message>
Restore 1/2/4/8 scoring and add leaderboard validation tests.
Match the original pool point values, regenerate the Excel workbook and golden baseline for all 27 players, and lock in scores with comprehensive vitest coverage.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/NHL_Playoffs_2026_Bracket_Scorer.xlsx
+++ b/NHL_Playoffs_2026_Bracket_Scorer.xlsx
@@ -780,7 +780,7 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Round 1: 2 pts   Round 2: 4 pts   Conference Final: 6 pts   Stanley Cup Final: 10 pts   Correct games bonus: +1</t>
+          <t xml:space="preserve">   Round 1: 1 pt   Round 2: 2 pts   Conference Final: 4 pts   Stanley Cup Final: 8 pts   Correct games bonus: +1</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -7940,7 +7940,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -7950,7 +7950,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -7960,7 +7960,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">

</xml_diff>